<commit_message>
TMTT0005221 $ TMTT0011420, Changes mar 14 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0011419_VerifyTASSupervisorCanonlyEnterLessThan24HoursForOneDayforAssociatesLightningView.xlsx
+++ b/TestData/LV_TMTT0011419_VerifyTASSupervisorCanonlyEnterLessThan24HoursForOneDayforAssociatesLightningView.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454DB34A-6966-4E3E-BEAC-0EAD0066D3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB89C829-E49A-4AA1-AAD3-4011BB9528FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="8" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Global Search User</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>Time Record Manager</t>
+  </si>
+  <si>
+    <t>115826</t>
   </si>
 </sst>
 </file>
@@ -882,26 +885,26 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -910,6 +913,9 @@
       </c>
       <c r="C2" t="s">
         <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TMTT0005430, TMTI0045469, TMTI0045470 Mar 15 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0011419_VerifyTASSupervisorCanonlyEnterLessThan24HoursForOneDayforAssociatesLightningView.xlsx
+++ b/TestData/LV_TMTT0011419_VerifyTASSupervisorCanonlyEnterLessThan24HoursForOneDayforAssociatesLightningView.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB89C829-E49A-4AA1-AAD3-4011BB9528FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0052049-B48D-4DF6-BDC6-109F6E44E56E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="8" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>Global Search User</t>
   </si>
@@ -111,6 +111,18 @@
   </si>
   <si>
     <t>115826</t>
+  </si>
+  <si>
+    <t>Time Tracking Beta Supervisor</t>
+  </si>
+  <si>
+    <t>GroupNam</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>CAO</t>
   </si>
 </sst>
 </file>
@@ -819,34 +831,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BA9779A-E3DE-42CF-890B-727C0A1D4E98}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BA9779A-E3DE-42CF-890B-727C0A1D4E98}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>